<commit_message>
Betonforløb lagt ud - videre med CA.
</commit_message>
<xml_diff>
--- a/undervisningsforlob/cambridge_analytica/data/social_media_openness_content_dataset.xlsx
+++ b/undervisningsforlob/cambridge_analytica/data/social_media_openness_content_dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\Documents\GitHub\aalborg-intelligence.github.io\undervisningsforlob\cambridge_analytica\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E9C0B9-5C0A-40E1-B20F-13BB6318BA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E7260A-F92B-418A-BED7-995CD7C93C67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="15670" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5568" yWindow="1044" windowWidth="30960" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -421,9 +421,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G301"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.6640625" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" customWidth="1"/>
+    <col min="5" max="5" width="18.21875" customWidth="1"/>
+    <col min="6" max="6" width="21.109375" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -446,7 +455,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>32</v>
       </c>
@@ -469,7 +478,7 @@
         <v>0.53900000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>29</v>
       </c>
@@ -492,7 +501,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>17</v>
       </c>
@@ -515,7 +524,7 @@
         <v>0.26100000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>23</v>
       </c>
@@ -538,7 +547,7 @@
         <v>0.41</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>23</v>
       </c>
@@ -561,7 +570,7 @@
         <v>0.14099999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>29</v>
       </c>
@@ -584,7 +593,7 @@
         <v>0.38500000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>17</v>
       </c>
@@ -607,7 +616,7 @@
         <v>0.251</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>30</v>
       </c>
@@ -630,7 +639,7 @@
         <v>0.52100000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>24</v>
       </c>
@@ -653,7 +662,7 @@
         <v>0.28699999999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>18</v>
       </c>
@@ -676,7 +685,7 @@
         <v>0.376</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>22</v>
       </c>
@@ -699,7 +708,7 @@
         <v>0.20699999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
@@ -722,7 +731,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>22</v>
       </c>
@@ -745,7 +754,7 @@
         <v>0.312</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>34</v>
       </c>
@@ -768,7 +777,7 @@
         <v>0.55700000000000005</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>32</v>
       </c>
@@ -791,7 +800,7 @@
         <v>0.57899999999999996</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>25</v>
       </c>
@@ -814,7 +823,7 @@
         <v>0.35099999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>27</v>
       </c>
@@ -837,7 +846,7 @@
         <v>0.373</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -860,7 +869,7 @@
         <v>0.36099999999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>23</v>
       </c>
@@ -883,7 +892,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>24</v>
       </c>
@@ -906,7 +915,7 @@
         <v>0.31900000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>24</v>
       </c>
@@ -929,7 +938,7 @@
         <v>0.61599999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
@@ -952,7 +961,7 @@
         <v>0.42199999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>31</v>
       </c>
@@ -975,7 +984,7 @@
         <v>0.46800000000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>21</v>
       </c>
@@ -1021,7 +1030,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>29</v>
       </c>
@@ -1044,7 +1053,7 @@
         <v>0.55500000000000005</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>20</v>
       </c>
@@ -1067,7 +1076,7 @@
         <v>0.35099999999999998</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>31</v>
       </c>
@@ -1090,7 +1099,7 @@
         <v>0.52200000000000002</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
@@ -1113,7 +1122,7 @@
         <v>0.59499999999999997</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>22</v>
       </c>
@@ -1136,7 +1145,7 @@
         <v>0.63300000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -1159,7 +1168,7 @@
         <v>0.56499999999999995</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>27</v>
       </c>
@@ -1182,7 +1191,7 @@
         <v>0.308</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>25</v>
       </c>
@@ -1205,7 +1214,7 @@
         <v>0.35199999999999998</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>28</v>
       </c>
@@ -1228,7 +1237,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>19</v>
       </c>
@@ -1251,7 +1260,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>27</v>
       </c>
@@ -1274,7 +1283,7 @@
         <v>0.29699999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>26</v>
       </c>
@@ -1297,7 +1306,7 @@
         <v>0.51700000000000002</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>29</v>
       </c>
@@ -1320,7 +1329,7 @@
         <v>0.36499999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>21</v>
       </c>
@@ -1343,7 +1352,7 @@
         <v>0.28899999999999998</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>24</v>
       </c>
@@ -1366,7 +1375,7 @@
         <v>0.34599999999999997</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>34</v>
       </c>
@@ -1389,7 +1398,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>21</v>
       </c>
@@ -1412,7 +1421,7 @@
         <v>0.26800000000000002</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>22</v>
       </c>
@@ -1435,7 +1444,7 @@
         <v>0.224</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>28</v>
       </c>
@@ -1458,7 +1467,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>33</v>
       </c>
@@ -1481,7 +1490,7 @@
         <v>0.57699999999999996</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>24</v>
       </c>
@@ -1504,7 +1513,7 @@
         <v>0.28699999999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>22</v>
       </c>
@@ -1527,7 +1536,7 @@
         <v>0.57499999999999996</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>21</v>
       </c>
@@ -1550,7 +1559,7 @@
         <v>0.17299999999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>21</v>
       </c>
@@ -1573,7 +1582,7 @@
         <v>0.52400000000000002</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>31</v>
       </c>
@@ -1596,7 +1605,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>21</v>
       </c>
@@ -1619,7 +1628,7 @@
         <v>0.374</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>32</v>
       </c>
@@ -1642,7 +1651,7 @@
         <v>0.47099999999999997</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>25</v>
       </c>
@@ -1665,7 +1674,7 @@
         <v>0.32900000000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>25</v>
       </c>
@@ -1688,7 +1697,7 @@
         <v>0.28899999999999998</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>25</v>
       </c>
@@ -1711,7 +1720,7 @@
         <v>0.53100000000000003</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>18</v>
       </c>
@@ -1734,7 +1743,7 @@
         <v>0.314</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>24</v>
       </c>
@@ -1757,7 +1766,7 @@
         <v>0.44800000000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>31</v>
       </c>
@@ -1780,7 +1789,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>30</v>
       </c>
@@ -1803,7 +1812,7 @@
         <v>0.30099999999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>27</v>
       </c>
@@ -1826,7 +1835,7 @@
         <v>0.41599999999999998</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>23</v>
       </c>
@@ -1849,7 +1858,7 @@
         <v>0.309</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>25</v>
       </c>
@@ -1872,7 +1881,7 @@
         <v>0.36899999999999999</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>25</v>
       </c>
@@ -1895,7 +1904,7 @@
         <v>0.48199999999999998</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>25</v>
       </c>
@@ -1918,7 +1927,7 @@
         <v>0.42399999999999999</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>29</v>
       </c>
@@ -1941,7 +1950,7 @@
         <v>0.28499999999999998</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>22</v>
       </c>
@@ -1964,7 +1973,7 @@
         <v>0.51500000000000001</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>21</v>
       </c>
@@ -1987,7 +1996,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>26</v>
       </c>
@@ -2010,7 +2019,7 @@
         <v>0.46200000000000002</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>24</v>
       </c>
@@ -2033,7 +2042,7 @@
         <v>0.441</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>22</v>
       </c>
@@ -2056,7 +2065,7 @@
         <v>0.39700000000000002</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>21</v>
       </c>
@@ -2079,7 +2088,7 @@
         <v>0.55100000000000005</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>27</v>
       </c>
@@ -2102,7 +2111,7 @@
         <v>0.49199999999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>29</v>
       </c>
@@ -2125,7 +2134,7 @@
         <v>0.43099999999999999</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>18</v>
       </c>
@@ -2148,7 +2157,7 @@
         <v>0.40600000000000003</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>30</v>
       </c>
@@ -2171,7 +2180,7 @@
         <v>0.61199999999999999</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>23</v>
       </c>
@@ -2194,7 +2203,7 @@
         <v>0.222</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>20</v>
       </c>
@@ -2217,7 +2226,7 @@
         <v>0.32700000000000001</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>20</v>
       </c>
@@ -2240,7 +2249,7 @@
         <v>0.56299999999999994</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>28</v>
       </c>
@@ -2263,7 +2272,7 @@
         <v>0.40200000000000002</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>26</v>
       </c>
@@ -2286,7 +2295,7 @@
         <v>0.72699999999999998</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>23</v>
       </c>
@@ -2309,7 +2318,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>23</v>
       </c>
@@ -2332,7 +2341,7 @@
         <v>0.183</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>26</v>
       </c>
@@ -2355,7 +2364,7 @@
         <v>0.55600000000000005</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>24</v>
       </c>
@@ -2378,7 +2387,7 @@
         <v>0.377</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>23</v>
       </c>
@@ -2401,7 +2410,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>28</v>
       </c>
@@ -2424,7 +2433,7 @@
         <v>0.46800000000000003</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>32</v>
       </c>
@@ -2447,7 +2456,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>28</v>
       </c>
@@ -2470,7 +2479,7 @@
         <v>0.33500000000000002</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>27</v>
       </c>
@@ -2493,7 +2502,7 @@
         <v>0.434</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>25</v>
       </c>
@@ -2516,7 +2525,7 @@
         <v>0.36899999999999999</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>17</v>
       </c>
@@ -2539,7 +2548,7 @@
         <v>0.41</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>16</v>
       </c>
@@ -2562,7 +2571,7 @@
         <v>0.35499999999999998</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>25</v>
       </c>
@@ -2585,7 +2594,7 @@
         <v>0.313</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>31</v>
       </c>
@@ -2608,7 +2617,7 @@
         <v>0.44900000000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>16</v>
       </c>
@@ -2631,7 +2640,7 @@
         <v>0.192</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>24</v>
       </c>
@@ -2654,7 +2663,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>24</v>
       </c>
@@ -2677,7 +2686,7 @@
         <v>0.55900000000000005</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>15</v>
       </c>
@@ -2700,7 +2709,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>19</v>
       </c>
@@ -2723,7 +2732,7 @@
         <v>0.316</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>24</v>
       </c>
@@ -2746,7 +2755,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>20</v>
       </c>
@@ -2769,7 +2778,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>25</v>
       </c>
@@ -2792,7 +2801,7 @@
         <v>0.33500000000000002</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>12</v>
       </c>
@@ -2815,7 +2824,7 @@
         <v>0.33800000000000002</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>22</v>
       </c>
@@ -2838,7 +2847,7 @@
         <v>0.29199999999999998</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>23</v>
       </c>
@@ -2861,7 +2870,7 @@
         <v>0.36499999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>33</v>
       </c>
@@ -2884,7 +2893,7 @@
         <v>0.33800000000000002</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>23</v>
       </c>
@@ -2907,7 +2916,7 @@
         <v>0.36599999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>24</v>
       </c>
@@ -2930,7 +2939,7 @@
         <v>0.47699999999999998</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>28</v>
       </c>
@@ -2953,7 +2962,7 @@
         <v>0.47599999999999998</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>23</v>
       </c>
@@ -2976,7 +2985,7 @@
         <v>0.313</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>22</v>
       </c>
@@ -2999,7 +3008,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>34</v>
       </c>
@@ -3022,7 +3031,7 @@
         <v>0.51400000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>28</v>
       </c>
@@ -3045,7 +3054,7 @@
         <v>0.34799999999999998</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>27</v>
       </c>
@@ -3068,7 +3077,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>24</v>
       </c>
@@ -3091,7 +3100,7 @@
         <v>0.27600000000000002</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>20</v>
       </c>
@@ -3114,7 +3123,7 @@
         <v>0.311</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>16</v>
       </c>
@@ -3137,7 +3146,7 @@
         <v>0.36199999999999999</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>29</v>
       </c>
@@ -3160,7 +3169,7 @@
         <v>0.39300000000000002</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>29</v>
       </c>
@@ -3183,7 +3192,7 @@
         <v>0.48599999999999999</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>19</v>
       </c>
@@ -3206,7 +3215,7 @@
         <v>0.41499999999999998</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>22</v>
       </c>
@@ -3229,7 +3238,7 @@
         <v>0.41299999999999998</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>23</v>
       </c>
@@ -3252,7 +3261,7 @@
         <v>0.28299999999999997</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>31</v>
       </c>
@@ -3275,7 +3284,7 @@
         <v>0.38300000000000001</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>12</v>
       </c>
@@ -3298,7 +3307,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>27</v>
       </c>
@@ -3321,7 +3330,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>17</v>
       </c>
@@ -3344,7 +3353,7 @@
         <v>0.39600000000000002</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>30</v>
       </c>
@@ -3367,7 +3376,7 @@
         <v>0.44800000000000001</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>27</v>
       </c>
@@ -3390,7 +3399,7 @@
         <v>0.48599999999999999</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>26</v>
       </c>
@@ -3413,7 +3422,7 @@
         <v>0.44600000000000001</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>31</v>
       </c>
@@ -3436,7 +3445,7 @@
         <v>0.36599999999999999</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>20</v>
       </c>
@@ -3459,7 +3468,7 @@
         <v>0.20499999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>19</v>
       </c>
@@ -3482,7 +3491,7 @@
         <v>0.224</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>29</v>
       </c>
@@ -3505,7 +3514,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>25</v>
       </c>
@@ -3528,7 +3537,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>27</v>
       </c>
@@ -3551,7 +3560,7 @@
         <v>0.52700000000000002</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>21</v>
       </c>
@@ -3574,7 +3583,7 @@
         <v>0.48099999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>20</v>
       </c>
@@ -3597,7 +3606,7 @@
         <v>0.437</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>23</v>
       </c>
@@ -3620,7 +3629,7 @@
         <v>0.47199999999999998</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>22</v>
       </c>
@@ -3643,7 +3652,7 @@
         <v>0.42399999999999999</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>30</v>
       </c>
@@ -3666,7 +3675,7 @@
         <v>0.48199999999999998</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>20</v>
       </c>
@@ -3689,7 +3698,7 @@
         <v>0.57599999999999996</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>21</v>
       </c>
@@ -3712,7 +3721,7 @@
         <v>0.54800000000000004</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>16</v>
       </c>
@@ -3735,7 +3744,7 @@
         <v>0.36399999999999999</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>22</v>
       </c>
@@ -3758,7 +3767,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>33</v>
       </c>
@@ -3781,7 +3790,7 @@
         <v>0.36699999999999999</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>23</v>
       </c>
@@ -3804,7 +3813,7 @@
         <v>0.41099999999999998</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>25</v>
       </c>
@@ -3827,7 +3836,7 @@
         <v>0.45900000000000002</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>30</v>
       </c>
@@ -3850,7 +3859,7 @@
         <v>0.50600000000000001</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>21</v>
       </c>
@@ -3873,7 +3882,7 @@
         <v>0.38500000000000001</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>26</v>
       </c>
@@ -3896,7 +3905,7 @@
         <v>0.56899999999999995</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>27</v>
       </c>
@@ -3919,7 +3928,7 @@
         <v>0.34399999999999997</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>32</v>
       </c>
@@ -3942,7 +3951,7 @@
         <v>0.45900000000000002</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>25</v>
       </c>
@@ -3965,7 +3974,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>21</v>
       </c>
@@ -3988,7 +3997,7 @@
         <v>0.374</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>29</v>
       </c>
@@ -4011,7 +4020,7 @@
         <v>0.437</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>29</v>
       </c>
@@ -4034,7 +4043,7 @@
         <v>0.35799999999999998</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>17</v>
       </c>
@@ -4057,7 +4066,7 @@
         <v>0.44400000000000001</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>27</v>
       </c>
@@ -4080,7 +4089,7 @@
         <v>0.42199999999999999</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>18</v>
       </c>
@@ -4103,7 +4112,7 @@
         <v>0.13600000000000001</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>25</v>
       </c>
@@ -4126,7 +4135,7 @@
         <v>0.54800000000000004</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>20</v>
       </c>
@@ -4149,7 +4158,7 @@
         <v>0.29899999999999999</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>27</v>
       </c>
@@ -4172,7 +4181,7 @@
         <v>0.34200000000000003</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>29</v>
       </c>
@@ -4195,7 +4204,7 @@
         <v>0.40699999999999997</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>23</v>
       </c>
@@ -4218,7 +4227,7 @@
         <v>0.16400000000000001</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>22</v>
       </c>
@@ -4241,7 +4250,7 @@
         <v>0.23799999999999999</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>34</v>
       </c>
@@ -4264,7 +4273,7 @@
         <v>0.59299999999999997</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>24</v>
       </c>
@@ -4287,7 +4296,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>34</v>
       </c>
@@ -4310,7 +4319,7 @@
         <v>0.53800000000000003</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>20</v>
       </c>
@@ -4333,7 +4342,7 @@
         <v>0.36399999999999999</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>26</v>
       </c>
@@ -4356,7 +4365,7 @@
         <v>0.34399999999999997</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>25</v>
       </c>
@@ -4379,7 +4388,7 @@
         <v>0.46100000000000002</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>18</v>
       </c>
@@ -4402,7 +4411,7 @@
         <v>0.27400000000000002</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>14</v>
       </c>
@@ -4425,7 +4434,7 @@
         <v>0.191</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>34</v>
       </c>
@@ -4448,7 +4457,7 @@
         <v>0.36499999999999999</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>26</v>
       </c>
@@ -4471,7 +4480,7 @@
         <v>0.51300000000000001</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>31</v>
       </c>
@@ -4494,7 +4503,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>11</v>
       </c>
@@ -4517,7 +4526,7 @@
         <v>0.17199999999999999</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>30</v>
       </c>
@@ -4540,7 +4549,7 @@
         <v>0.44500000000000001</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>23</v>
       </c>
@@ -4563,7 +4572,7 @@
         <v>0.39900000000000002</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>30</v>
       </c>
@@ -4586,7 +4595,7 @@
         <v>0.501</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>32</v>
       </c>
@@ -4609,7 +4618,7 @@
         <v>0.499</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>23</v>
       </c>
@@ -4632,7 +4641,7 @@
         <v>0.20799999999999999</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>18</v>
       </c>
@@ -4655,7 +4664,7 @@
         <v>0.432</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>29</v>
       </c>
@@ -4678,7 +4687,7 @@
         <v>0.377</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>22</v>
       </c>
@@ -4701,7 +4710,7 @@
         <v>0.33200000000000002</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>34</v>
       </c>
@@ -4724,7 +4733,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>28</v>
       </c>
@@ -4747,7 +4756,7 @@
         <v>0.61599999999999999</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>25</v>
       </c>
@@ -4770,7 +4779,7 @@
         <v>0.63100000000000001</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>29</v>
       </c>
@@ -4793,7 +4802,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>35</v>
       </c>
@@ -4816,7 +4825,7 @@
         <v>0.39900000000000002</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>26</v>
       </c>
@@ -4839,7 +4848,7 @@
         <v>0.36599999999999999</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>26</v>
       </c>
@@ -4862,7 +4871,7 @@
         <v>0.48099999999999998</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>20</v>
       </c>
@@ -4885,7 +4894,7 @@
         <v>0.247</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>24</v>
       </c>
@@ -4908,7 +4917,7 @@
         <v>0.34300000000000003</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>21</v>
       </c>
@@ -4931,7 +4940,7 @@
         <v>0.22800000000000001</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>25</v>
       </c>
@@ -4954,7 +4963,7 @@
         <v>0.23200000000000001</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>16</v>
       </c>
@@ -4977,7 +4986,7 @@
         <v>0.30199999999999999</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>25</v>
       </c>
@@ -5000,7 +5009,7 @@
         <v>0.56299999999999994</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>22</v>
       </c>
@@ -5023,7 +5032,7 @@
         <v>0.376</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>23</v>
       </c>
@@ -5046,7 +5055,7 @@
         <v>0.182</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>31</v>
       </c>
@@ -5069,7 +5078,7 @@
         <v>0.621</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>30</v>
       </c>
@@ -5092,7 +5101,7 @@
         <v>0.502</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>31</v>
       </c>
@@ -5115,7 +5124,7 @@
         <v>0.42199999999999999</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>21</v>
       </c>
@@ -5138,7 +5147,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>22</v>
       </c>
@@ -5161,7 +5170,7 @@
         <v>0.34899999999999998</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>25</v>
       </c>
@@ -5184,7 +5193,7 @@
         <v>0.30299999999999999</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>25</v>
       </c>
@@ -5207,7 +5216,7 @@
         <v>0.38300000000000001</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>19</v>
       </c>
@@ -5230,7 +5239,7 @@
         <v>0.34300000000000003</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>25</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>0.224</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>22</v>
       </c>
@@ -5276,7 +5285,7 @@
         <v>0.41399999999999998</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>26</v>
       </c>
@@ -5299,7 +5308,7 @@
         <v>0.36799999999999999</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>27</v>
       </c>
@@ -5322,7 +5331,7 @@
         <v>0.48399999999999999</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>26</v>
       </c>
@@ -5345,7 +5354,7 @@
         <v>0.38200000000000001</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>20</v>
       </c>
@@ -5368,7 +5377,7 @@
         <v>0.24299999999999999</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>20</v>
       </c>
@@ -5391,7 +5400,7 @@
         <v>0.38100000000000001</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>28</v>
       </c>
@@ -5414,7 +5423,7 @@
         <v>0.50700000000000001</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>19</v>
       </c>
@@ -5437,7 +5446,7 @@
         <v>0.46600000000000003</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>24</v>
       </c>
@@ -5460,7 +5469,7 @@
         <v>0.441</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>23</v>
       </c>
@@ -5483,7 +5492,7 @@
         <v>0.19500000000000001</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>21</v>
       </c>
@@ -5506,7 +5515,7 @@
         <v>0.28100000000000003</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>23</v>
       </c>
@@ -5529,7 +5538,7 @@
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>18</v>
       </c>
@@ -5552,7 +5561,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>22</v>
       </c>
@@ -5575,7 +5584,7 @@
         <v>0.29799999999999999</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>27</v>
       </c>
@@ -5598,7 +5607,7 @@
         <v>0.34200000000000003</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>28</v>
       </c>
@@ -5621,7 +5630,7 @@
         <v>0.46200000000000002</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>15</v>
       </c>
@@ -5644,7 +5653,7 @@
         <v>0.28599999999999998</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>22</v>
       </c>
@@ -5667,7 +5676,7 @@
         <v>0.39400000000000002</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>23</v>
       </c>
@@ -5690,7 +5699,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>18</v>
       </c>
@@ -5713,7 +5722,7 @@
         <v>0.32100000000000001</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>33</v>
       </c>
@@ -5736,7 +5745,7 @@
         <v>0.48399999999999999</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>22</v>
       </c>
@@ -5759,7 +5768,7 @@
         <v>0.245</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>21</v>
       </c>
@@ -5782,7 +5791,7 @@
         <v>0.34499999999999997</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>31</v>
       </c>
@@ -5805,7 +5814,7 @@
         <v>0.59499999999999997</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>28</v>
       </c>
@@ -5828,7 +5837,7 @@
         <v>0.35799999999999998</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>22</v>
       </c>
@@ -5851,7 +5860,7 @@
         <v>0.372</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>14</v>
       </c>
@@ -5874,7 +5883,7 @@
         <v>0.36399999999999999</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>34</v>
       </c>
@@ -5897,7 +5906,7 @@
         <v>0.48399999999999999</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>33</v>
       </c>
@@ -5920,7 +5929,7 @@
         <v>0.53500000000000003</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>23</v>
       </c>
@@ -5943,7 +5952,7 @@
         <v>0.26100000000000001</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>28</v>
       </c>
@@ -5966,7 +5975,7 @@
         <v>0.253</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>28</v>
       </c>
@@ -5989,7 +5998,7 @@
         <v>0.41699999999999998</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>26</v>
       </c>
@@ -6012,7 +6021,7 @@
         <v>0.66900000000000004</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>20</v>
       </c>
@@ -6035,7 +6044,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>14</v>
       </c>
@@ -6058,7 +6067,7 @@
         <v>0.245</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>21</v>
       </c>
@@ -6081,7 +6090,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>19</v>
       </c>
@@ -6104,7 +6113,7 @@
         <v>0.52400000000000002</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>29</v>
       </c>
@@ -6127,7 +6136,7 @@
         <v>0.52200000000000002</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>19</v>
       </c>
@@ -6150,7 +6159,7 @@
         <v>0.11700000000000001</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>17</v>
       </c>
@@ -6173,7 +6182,7 @@
         <v>0.371</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>28</v>
       </c>
@@ -6196,7 +6205,7 @@
         <v>0.59199999999999997</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>19</v>
       </c>
@@ -6219,7 +6228,7 @@
         <v>0.20200000000000001</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>25</v>
       </c>
@@ -6242,7 +6251,7 @@
         <v>0.36199999999999999</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>24</v>
       </c>
@@ -6265,7 +6274,7 @@
         <v>0.53200000000000003</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>23</v>
       </c>
@@ -6288,7 +6297,7 @@
         <v>0.40699999999999997</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>22</v>
       </c>
@@ -6311,7 +6320,7 @@
         <v>0.33900000000000002</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>27</v>
       </c>
@@ -6334,7 +6343,7 @@
         <v>0.55500000000000005</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>21</v>
       </c>
@@ -6357,7 +6366,7 @@
         <v>0.28599999999999998</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>26</v>
       </c>
@@ -6380,7 +6389,7 @@
         <v>0.67200000000000004</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>28</v>
       </c>
@@ -6403,7 +6412,7 @@
         <v>0.48499999999999999</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>25</v>
       </c>
@@ -6426,7 +6435,7 @@
         <v>0.36899999999999999</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>20</v>
       </c>
@@ -6449,7 +6458,7 @@
         <v>0.24299999999999999</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>20</v>
       </c>
@@ -6472,7 +6481,7 @@
         <v>0.313</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>30</v>
       </c>
@@ -6495,7 +6504,7 @@
         <v>0.26900000000000002</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>26</v>
       </c>
@@ -6518,7 +6527,7 @@
         <v>0.38500000000000001</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>30</v>
       </c>
@@ -6541,7 +6550,7 @@
         <v>0.47699999999999998</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>24</v>
       </c>
@@ -6564,7 +6573,7 @@
         <v>0.45900000000000002</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>20</v>
       </c>
@@ -6587,7 +6596,7 @@
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>28</v>
       </c>
@@ -6610,7 +6619,7 @@
         <v>0.248</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>31</v>
       </c>
@@ -6633,7 +6642,7 @@
         <v>0.30199999999999999</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>20</v>
       </c>
@@ -6656,7 +6665,7 @@
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>26</v>
       </c>
@@ -6679,7 +6688,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>25</v>
       </c>
@@ -6702,7 +6711,7 @@
         <v>0.503</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>36</v>
       </c>
@@ -6725,7 +6734,7 @@
         <v>0.53700000000000003</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>25</v>
       </c>
@@ -6748,7 +6757,7 @@
         <v>0.41399999999999998</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>25</v>
       </c>
@@ -6771,7 +6780,7 @@
         <v>0.33700000000000002</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>32</v>
       </c>
@@ -6794,7 +6803,7 @@
         <v>0.621</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>26</v>
       </c>
@@ -6817,7 +6826,7 @@
         <v>0.46800000000000003</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>31</v>
       </c>
@@ -6840,7 +6849,7 @@
         <v>0.60299999999999998</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>18</v>
       </c>
@@ -6863,7 +6872,7 @@
         <v>0.219</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>18</v>
       </c>
@@ -6886,7 +6895,7 @@
         <v>0.44500000000000001</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>24</v>
       </c>
@@ -6909,7 +6918,7 @@
         <v>0.36399999999999999</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>35</v>
       </c>
@@ -6932,7 +6941,7 @@
         <v>0.58399999999999996</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>36</v>
       </c>
@@ -6955,7 +6964,7 @@
         <v>0.64600000000000002</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>18</v>
       </c>
@@ -6978,7 +6987,7 @@
         <v>0.158</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>19</v>
       </c>
@@ -7001,7 +7010,7 @@
         <v>0.40400000000000003</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>35</v>
       </c>
@@ -7024,7 +7033,7 @@
         <v>0.66900000000000004</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>23</v>
       </c>
@@ -7047,7 +7056,7 @@
         <v>0.59099999999999997</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>21</v>
       </c>
@@ -7070,7 +7079,7 @@
         <v>0.34100000000000003</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>28</v>
       </c>
@@ -7093,7 +7102,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>36</v>
       </c>
@@ -7116,7 +7125,7 @@
         <v>0.48199999999999998</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>26</v>
       </c>
@@ -7139,7 +7148,7 @@
         <v>0.47599999999999998</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>38</v>
       </c>
@@ -7162,7 +7171,7 @@
         <v>0.55500000000000005</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>20</v>
       </c>
@@ -7185,7 +7194,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>24</v>
       </c>
@@ -7208,7 +7217,7 @@
         <v>0.47099999999999997</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>24</v>
       </c>
@@ -7231,7 +7240,7 @@
         <v>0.28199999999999997</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>24</v>
       </c>
@@ -7254,7 +7263,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>32</v>
       </c>
@@ -7277,7 +7286,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>32</v>
       </c>
@@ -7300,7 +7309,7 @@
         <v>0.39500000000000002</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>23</v>
       </c>
@@ -7323,7 +7332,7 @@
         <v>0.26500000000000001</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>34</v>
       </c>

</xml_diff>